<commit_message>
Automation Toolkit Release v2024.3.0
</commit_message>
<xml_diff>
--- a/cd3_automation_toolkit/example/CD3-Blank-template.xlsx
+++ b/cd3_automation_toolkit/example/CD3-Blank-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susingla/PyCharmProjects/orahub-develop/cd3_automation_toolkit/example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19569292-BC0A-B14D-B0E7-0CBCFE65E647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE011F5-6BF6-964D-BE2C-54919FBFB3C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17420" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6940" yWindow="760" windowWidth="30240" windowHeight="17420" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Release-Info" sheetId="1" r:id="rId1"/>
@@ -373,7 +373,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Mansatory for Autotune Type - PERFORMANCE_BASED or BOTH</t>
+          <t>Mandatory for Autotune Type - PERFORMANCE_BASED or BOTH</t>
         </r>
       </text>
     </comment>
@@ -382,30 +382,6 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Suruchi</author>
-  </authors>
-  <commentList>
-    <comment ref="L2" authorId="0" shapeId="0" xr:uid="{DFA3381A-B6E3-8642-9D9B-F59DB2F382DA}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Mansatory for Autotune Type - PERFORMANCE_BASED or BOTH</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Microsoft Office User</author>
@@ -650,7 +626,7 @@
 </comments>
 </file>
 
-<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Suruchi</author>
@@ -712,7 +688,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="775">
   <si>
     <t>Region</t>
   </si>
@@ -10327,12 +10303,318 @@
   <si>
     <t>Matching Rule</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Note:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Default value for columns if left blank: sourceCIDR- 0.0.0.0/0, Access- READ_WRITE, GID- 65534, UID- 65534, IDSquash- NONE and Require PS Port- false.
+Mount target IP will take default values from OCI if left blank.
+Resources will be created based on 'MountTarget Name' and 'FSS Name' columns.
+Below sample data shows example of  multiple FSS(FSS1 and FSS2) using single MT(MT1) , 1 FSS(FSS3) using multiple MTs(MT2 and MT3) and also 1 FSS(FSS4) using 1 MT(MT4).</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>onlyMT is Mount target without any FSS. onlyFSS is File System without any Mount Target or Export (used for replication)</t>
+    </r>
+  </si>
+  <si>
+    <t>MountTarget Name</t>
+  </si>
+  <si>
+    <t>MountTarget SubnetName</t>
+  </si>
+  <si>
+    <t>MountTarget IP</t>
+  </si>
+  <si>
+    <t>MountTarget Hostname</t>
+  </si>
+  <si>
+    <t>FSS Name</t>
+  </si>
+  <si>
+    <t>Source Snapshot</t>
+  </si>
+  <si>
+    <t>Snapshot Policy</t>
+  </si>
+  <si>
+    <t>Replication Information</t>
+  </si>
+  <si>
+    <t>Source CIDR</t>
+  </si>
+  <si>
+    <t>Access (READ_ONLY|READ_WRITE)</t>
+  </si>
+  <si>
+    <t>GID</t>
+  </si>
+  <si>
+    <t>UID</t>
+  </si>
+  <si>
+    <t>IDSquash (NONE|ALL|ROOT)</t>
+  </si>
+  <si>
+    <t>Require PS Port (true|false)</t>
+  </si>
+  <si>
+    <t>Is Anonymous Access Allowed</t>
+  </si>
+  <si>
+    <t>Allowed Auth</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"># Rows after &lt;END&gt; will not be processed (Sample data is provided for reference after &lt;END&gt;);
+Columns: Region, Compartment Name, Availability Domain, MountTarget Name, MountTarget SubnetName, FSS name, Path are mandatory.
+Freeform and Defined Tags - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>If specified, Applies to FSS object only and not to other components like Mount Target.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Enter subnet name as : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">vcn-name&gt;_&lt;subnet-name&gt;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Source Snapshot:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Accepts OCID of the source snapshot  or the name of the key defined under variable  fss_source_ocids in variables_&lt;region&gt;.tf file
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Snapshot Policy - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Accepts OCID of the snapshot policy or the name in format: &lt;snaphot_policy_compartment_name&gt;@&lt;snaphost_policy_name&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Replication Information: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Format - TargetFSS(OCID or Name)::ReplicationInterval::ReplicationName. Multiple replication values are seperated by newline in the same cell(\n is not supported). Ensure Target FSS for replication must not have exports created.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+"Defined Tags" - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Specify the defined tag key and its value in the format - &lt;Namespace&gt;.&lt;TagKey&gt;=&lt;Value&gt;  else leave it empty.
+                             Multiple Tag Key , Values can be specified using semi colon (;) as the delimiter. 
+                           </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Example: Operations.CostCenter=01;Users.Name=user01</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="44" x14ac:knownFonts="1">
+  <fonts count="45" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10658,6 +10940,15 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -10924,7 +11215,7 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -11203,6 +11494,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -22871,11 +23171,11 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.5" customWidth="1"/>
@@ -22887,8 +23187,8 @@
     <col min="8" max="8" width="8.5" customWidth="1"/>
     <col min="9" max="9" width="9.83203125" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="19.1640625" customWidth="1"/>
-    <col min="12" max="12" width="7.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
     <col min="13" max="13" width="8.5" customWidth="1"/>
     <col min="14" max="14" width="17.1640625" customWidth="1"/>
     <col min="15" max="15" width="15.5" customWidth="1"/>
@@ -22896,9 +23196,9 @@
     <col min="17" max="17" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="201" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" ht="169" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="97" t="s">
-        <v>749</v>
+        <v>774</v>
       </c>
       <c r="B1" s="98"/>
       <c r="C1" s="98"/>
@@ -22910,84 +23210,99 @@
       <c r="I1" s="98"/>
       <c r="J1" s="98"/>
       <c r="K1" s="98"/>
-      <c r="L1" s="98"/>
-      <c r="M1" s="98"/>
-      <c r="N1" s="98"/>
-      <c r="O1" s="98"/>
-      <c r="P1" s="98"/>
-      <c r="Q1" s="98"/>
-      <c r="R1" s="101"/>
-    </row>
-    <row r="2" spans="1:18" s="33" customFormat="1" ht="96" x14ac:dyDescent="0.2">
-      <c r="A2" s="25" t="s">
+      <c r="L1" s="101"/>
+      <c r="M1" s="113" t="s">
+        <v>757</v>
+      </c>
+      <c r="N1" s="114"/>
+      <c r="O1" s="114"/>
+      <c r="P1" s="114"/>
+      <c r="Q1" s="114"/>
+      <c r="R1" s="114"/>
+      <c r="S1" s="114"/>
+      <c r="T1" s="114"/>
+      <c r="U1" s="114"/>
+      <c r="V1" s="115"/>
+    </row>
+    <row r="2" spans="1:22" s="1" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" s="25" t="s">
-        <v>655</v>
-      </c>
-      <c r="E2" s="25" t="s">
-        <v>81</v>
+      <c r="C2" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>758</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>759</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>66</v>
+        <v>760</v>
       </c>
       <c r="G2" s="26" t="s">
-        <v>82</v>
+        <v>761</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>503</v>
+        <v>762</v>
       </c>
       <c r="J2" s="26" t="s">
-        <v>262</v>
+        <v>763</v>
       </c>
       <c r="K2" s="26" t="s">
-        <v>725</v>
+        <v>764</v>
       </c>
       <c r="L2" s="26" t="s">
-        <v>726</v>
+        <v>765</v>
       </c>
       <c r="M2" s="26" t="s">
-        <v>727</v>
+        <v>85</v>
       </c>
       <c r="N2" s="26" t="s">
-        <v>728</v>
+        <v>766</v>
       </c>
       <c r="O2" s="26" t="s">
-        <v>502</v>
+        <v>767</v>
       </c>
       <c r="P2" s="26" t="s">
-        <v>73</v>
+        <v>768</v>
       </c>
       <c r="Q2" s="26" t="s">
-        <v>377</v>
+        <v>769</v>
       </c>
       <c r="R2" s="26" t="s">
+        <v>770</v>
+      </c>
+      <c r="S2" s="26" t="s">
+        <v>771</v>
+      </c>
+      <c r="T2" s="26" t="s">
+        <v>772</v>
+      </c>
+      <c r="U2" s="26" t="s">
+        <v>773</v>
+      </c>
+      <c r="V2" s="26" t="s">
         <v>258</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:R1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="M1:V1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation allowBlank="1" sqref="A3:XFD1048576 A1:J2 L1:M2 O1:XFD2 N1" xr:uid="{02462EBB-6C3D-AD4C-90E1-0F01761ACD92}"/>
-    <dataValidation showInputMessage="1" showErrorMessage="1" sqref="N2" xr:uid="{44F44AA6-F9A2-F043-9A7C-E9C593C12245}"/>
-    <dataValidation type="list" sqref="K1:K2" xr:uid="{296BAB61-C7D2-7746-8608-28C808FD0978}">
-      <formula1>"BOTH,PERFORMANCE_BASED,DETACHED_VOLUME"</formula1>
-    </dataValidation>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" sqref="A3:XFD1048576 U1:XFD2 B2:L2 M1:S2 A1:A2" xr:uid="{02462EBB-6C3D-AD4C-90E1-0F01761ACD92}"/>
+    <dataValidation showInputMessage="1" showErrorMessage="1" sqref="T1:T2" xr:uid="{7A2F3F2A-4835-1545-9D47-36E98CCE349F}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -23585,15 +23900,15 @@
       <c r="J1" s="102" t="s">
         <v>267</v>
       </c>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="113"/>
-      <c r="O1" s="113"/>
-      <c r="P1" s="113"/>
-      <c r="Q1" s="113"/>
-      <c r="R1" s="113"/>
-      <c r="S1" s="114"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+      <c r="P1" s="116"/>
+      <c r="Q1" s="116"/>
+      <c r="R1" s="116"/>
+      <c r="S1" s="117"/>
     </row>
     <row r="2" spans="1:19" ht="58.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
@@ -31238,26 +31553,26 @@
       <c r="A1" s="108" t="s">
         <v>663</v>
       </c>
-      <c r="B1" s="115"/>
-      <c r="C1" s="115"/>
-      <c r="D1" s="115"/>
-      <c r="E1" s="115"/>
-      <c r="F1" s="115"/>
-      <c r="G1" s="115"/>
-      <c r="H1" s="115"/>
-      <c r="I1" s="115"/>
-      <c r="J1" s="115"/>
-      <c r="K1" s="115"/>
-      <c r="L1" s="115"/>
-      <c r="M1" s="115"/>
-      <c r="N1" s="115"/>
-      <c r="O1" s="115"/>
-      <c r="P1" s="115"/>
-      <c r="Q1" s="115"/>
-      <c r="R1" s="115"/>
-      <c r="S1" s="115"/>
-      <c r="T1" s="115"/>
-      <c r="U1" s="115"/>
+      <c r="B1" s="118"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
+      <c r="I1" s="118"/>
+      <c r="J1" s="118"/>
+      <c r="K1" s="118"/>
+      <c r="L1" s="118"/>
+      <c r="M1" s="118"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="118"/>
+      <c r="P1" s="118"/>
+      <c r="Q1" s="118"/>
+      <c r="R1" s="118"/>
+      <c r="S1" s="118"/>
+      <c r="T1" s="118"/>
+      <c r="U1" s="118"/>
       <c r="V1" s="60"/>
       <c r="W1" s="60"/>
       <c r="X1" s="60"/>
@@ -35563,26 +35878,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="138" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="119" t="s">
         <v>710</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="118"/>
+      <c r="B1" s="120"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
+      <c r="F1" s="120"/>
+      <c r="G1" s="120"/>
+      <c r="H1" s="120"/>
+      <c r="I1" s="120"/>
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="121"/>
     </row>
     <row r="2" spans="1:18" s="40" customFormat="1" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="26" t="s">
@@ -35802,26 +36117,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="261" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="122" t="s">
         <v>687</v>
       </c>
-      <c r="B1" s="120"/>
-      <c r="C1" s="120"/>
-      <c r="D1" s="120"/>
-      <c r="E1" s="120"/>
-      <c r="F1" s="120"/>
-      <c r="G1" s="120"/>
-      <c r="H1" s="120"/>
-      <c r="I1" s="120"/>
-      <c r="J1" s="120"/>
-      <c r="K1" s="120"/>
-      <c r="L1" s="120"/>
-      <c r="M1" s="120"/>
-      <c r="N1" s="120"/>
-      <c r="O1" s="120"/>
-      <c r="P1" s="120"/>
-      <c r="Q1" s="120"/>
-      <c r="R1" s="121"/>
+      <c r="B1" s="123"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
+      <c r="E1" s="123"/>
+      <c r="F1" s="123"/>
+      <c r="G1" s="123"/>
+      <c r="H1" s="123"/>
+      <c r="I1" s="123"/>
+      <c r="J1" s="123"/>
+      <c r="K1" s="123"/>
+      <c r="L1" s="123"/>
+      <c r="M1" s="123"/>
+      <c r="N1" s="123"/>
+      <c r="O1" s="123"/>
+      <c r="P1" s="123"/>
+      <c r="Q1" s="123"/>
+      <c r="R1" s="124"/>
     </row>
     <row r="2" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="s">

</xml_diff>

<commit_message>
Automation Toolkit Release v2025.2.0
</commit_message>
<xml_diff>
--- a/cd3_automation_toolkit/example/CD3-Blank-template.xlsx
+++ b/cd3_automation_toolkit/example/CD3-Blank-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10921"/>
   <workbookPr updateLinks="never" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susingla/PyCharmProjects/orahub-develop1/cd3_automation_toolkit/example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF558CF2-22C7-C644-BF37-9285823665BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46525C24-A1D3-F24E-95B3-6B7855813156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="220" yWindow="1080" windowWidth="30240" windowHeight="17480" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5685,198 +5685,6 @@
     <t>Alert Message</t>
   </si>
   <si>
-    <r>
-      <t># Rows after &lt;END&gt; will not be processed (Sample data is provided for reference after &lt;END&gt;);
-All fields are mandatory for each VCN except "DNS Label" and "Defined Tag".
-Tags apply to the VCNs only and not to its components like IGW,NGW,SGW,DRG,LPG.
-"VCN name"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> -  VCN names should be unique and are case-sensitie across sheets.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"CIDR Blocks" </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>- Enter comma seperated CIDRs to have multiple CIDR blocks attached to VCN.
-"</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>DNS Label"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> -  Default value is "VCN Name" truncated to 15 chars (when left empty).If specified as </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>'n'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, DNS will not be enabled for the VCN.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Valid Values for columns E,F,G,H - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>y|n|&lt;component_name&gt; i.e. specify 'n' when a component(like IGW) is 
-                                                                    not required to be configured(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>eg:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> PHXHub-VCN in sample data), 
-                                                                 - specify name of the component- component will be configured with the
-                                                                    mentioned name(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>eg:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> PHX-DRG for the DRG in PHXHub-VCN) ,
-                                                                 - specify 'y' if component needs to be configured with default name i.e. 
-                                                                    &lt;vcnname&gt;_ngw(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>eg:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> PHXNonProd-VCN_ngw)
-                                                    </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Calibri (Body)"/>
-      </rPr>
-      <t>Route Table associated with DRG/IGW/NGW/SGW can be specified in below format:
-                                                    y::&lt;Route Table Name&gt; or &lt;component_name::&lt;Route Table Name&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
     <t>Autotune Type</t>
   </si>
   <si>
@@ -11137,51 +10945,6 @@
     <t>Singapore-2</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CD3 Automation Toolkit</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Release - v2025.2.0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Updated ADB sheet, VCNs sheet</t>
-    </r>
-  </si>
-  <si>
     <t>Oracle GUA IPv6 Enabled</t>
   </si>
   <si>
@@ -11435,6 +11198,243 @@
   </si>
   <si>
     <t>Data Storage Size</t>
+  </si>
+  <si>
+    <r>
+      <t># Rows after &lt;END&gt; will not be processed (Sample data is provided for reference after &lt;END&gt;);
+All fields are mandatory for each VCN except "DNS Label" and "Defined Tag".
+Tags apply to the VCNs only and not to its components like IGW,NGW,SGW,DRG,LPG.
+"VCN name"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -  VCN names should be unique and are case-sensitie across sheets.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"CIDR Blocks" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Enter comma seperated CIDRs to have multiple CIDR blocks attached to VCN.
+"</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DNS Label"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -  Default value is "VCN Name" truncated to 15 chars (when left empty).If specified as </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'n'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, DNS will not be enabled for the VCN.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Valid Values for columns H, I, J, K, L - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>y|n|&lt;component_name&gt; i.e. specify 'n' when a component(like IGW) is 
+                                                                    not required to be configured(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>eg:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> PHXHub-VCN in sample data), 
+                                                                 - specify name of the component- component will be configured with the
+                                                                    mentioned name(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>eg:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> PHX-DRG for the DRG in PHXHub-VCN) ,
+                                                                 - specify 'y' if component needs to be configured with default name i.e. 
+                                                                    &lt;vcnname&gt;_ngw(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>eg:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> PHXNonProd-VCN_ngw)
+                                                    </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>Route Table associated with DRG/IGW/NGW/SGW can be specified in below format:
+                                                    y::&lt;Route Table Name&gt; or &lt;component_name::&lt;Route Table Name&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CD3 Automation Toolkit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Release - v2025.2.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Updated ADB sheet, VCNs sheet, Groups and Policies as per CIS LZ</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -17598,7 +17598,7 @@
     <row r="1" spans="1:1" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:1" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="57" t="s">
-        <v>796</v>
+        <v>806</v>
       </c>
     </row>
   </sheetData>
@@ -17633,7 +17633,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="247" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="103" t="s">
-        <v>693</v>
+        <v>805</v>
       </c>
       <c r="B1" s="104"/>
       <c r="C1" s="104"/>
@@ -17644,7 +17644,7 @@
       <c r="H1" s="104"/>
       <c r="I1" s="105"/>
       <c r="J1" s="103" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="K1" s="104"/>
       <c r="L1" s="104"/>
@@ -17666,13 +17666,13 @@
         <v>484</v>
       </c>
       <c r="E2" s="15" t="s">
+        <v>795</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>796</v>
+      </c>
+      <c r="G2" s="15" t="s">
         <v>797</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>798</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>799</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>12</v>
@@ -17738,7 +17738,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="222" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -17812,7 +17812,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="30" customFormat="1" ht="94" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B1" s="108"/>
     </row>
@@ -17878,7 +17878,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="136" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -18006,7 +18006,7 @@
         <v>11</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="H2" s="25" t="s">
         <v>29</v>
@@ -23883,7 +23883,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="226" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="114" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B1" s="115"/>
       <c r="C1" s="115"/>
@@ -23893,7 +23893,7 @@
       <c r="G1" s="115"/>
       <c r="H1" s="116"/>
       <c r="I1" s="103" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="J1" s="104"/>
       <c r="K1" s="104"/>
@@ -23926,7 +23926,7 @@
         <v>67</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="G2" s="24" t="s">
         <v>69</v>
@@ -24016,7 +24016,7 @@
   <sheetData>
     <row r="1" spans="1:18" ht="201" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="103" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B1" s="104"/>
       <c r="C1" s="104"/>
@@ -24068,16 +24068,16 @@
         <v>258</v>
       </c>
       <c r="K2" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="L2" s="25" t="s">
         <v>694</v>
       </c>
-      <c r="L2" s="25" t="s">
+      <c r="M2" s="25" t="s">
         <v>695</v>
       </c>
-      <c r="M2" s="25" t="s">
+      <c r="N2" s="25" t="s">
         <v>696</v>
-      </c>
-      <c r="N2" s="25" t="s">
-        <v>697</v>
       </c>
       <c r="O2" s="25" t="s">
         <v>495</v>
@@ -24141,7 +24141,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="169" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="103" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B1" s="104"/>
       <c r="C1" s="104"/>
@@ -24155,7 +24155,7 @@
       <c r="K1" s="104"/>
       <c r="L1" s="105"/>
       <c r="M1" s="117" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="N1" s="118"/>
       <c r="O1" s="118"/>
@@ -24178,58 +24178,58 @@
         <v>65</v>
       </c>
       <c r="D2" s="25" t="s">
+        <v>715</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>736</v>
+      </c>
+      <c r="F2" s="25" t="s">
         <v>716</v>
       </c>
-      <c r="E2" s="25" t="s">
-        <v>737</v>
-      </c>
-      <c r="F2" s="25" t="s">
+      <c r="G2" s="25" t="s">
         <v>717</v>
-      </c>
-      <c r="G2" s="25" t="s">
-        <v>718</v>
       </c>
       <c r="H2" s="25" t="s">
         <v>73</v>
       </c>
       <c r="I2" s="25" t="s">
+        <v>718</v>
+      </c>
+      <c r="J2" s="25" t="s">
         <v>719</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="K2" s="25" t="s">
         <v>720</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="L2" s="25" t="s">
         <v>721</v>
-      </c>
-      <c r="L2" s="25" t="s">
-        <v>722</v>
       </c>
       <c r="M2" s="25" t="s">
         <v>84</v>
       </c>
       <c r="N2" s="25" t="s">
+        <v>722</v>
+      </c>
+      <c r="O2" s="25" t="s">
         <v>723</v>
       </c>
-      <c r="O2" s="25" t="s">
+      <c r="P2" s="25" t="s">
         <v>724</v>
       </c>
-      <c r="P2" s="25" t="s">
+      <c r="Q2" s="25" t="s">
         <v>725</v>
       </c>
-      <c r="Q2" s="25" t="s">
+      <c r="R2" s="25" t="s">
         <v>726</v>
       </c>
-      <c r="R2" s="25" t="s">
+      <c r="S2" s="25" t="s">
         <v>727</v>
       </c>
-      <c r="S2" s="25" t="s">
+      <c r="T2" s="25" t="s">
         <v>728</v>
       </c>
-      <c r="T2" s="25" t="s">
+      <c r="U2" s="25" t="s">
         <v>729</v>
-      </c>
-      <c r="U2" s="25" t="s">
-        <v>730</v>
       </c>
       <c r="V2" s="25" t="s">
         <v>255</v>
@@ -24299,7 +24299,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="145" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="103" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B1" s="104"/>
       <c r="C1" s="104"/>
@@ -24316,7 +24316,7 @@
       <c r="N1" s="104"/>
       <c r="O1" s="105"/>
       <c r="P1" s="114" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="Q1" s="115"/>
       <c r="R1" s="115"/>
@@ -24361,10 +24361,10 @@
         <v>516</v>
       </c>
       <c r="H2" s="25" t="s">
+        <v>739</v>
+      </c>
+      <c r="I2" s="25" t="s">
         <v>740</v>
-      </c>
-      <c r="I2" s="25" t="s">
-        <v>741</v>
       </c>
       <c r="J2" s="25" t="s">
         <v>517</v>
@@ -24379,7 +24379,7 @@
         <v>520</v>
       </c>
       <c r="N2" s="25" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="O2" s="25" t="s">
         <v>521</v>
@@ -24403,7 +24403,7 @@
         <v>523</v>
       </c>
       <c r="V2" s="25" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="W2" s="25" t="s">
         <v>65</v>
@@ -24418,7 +24418,7 @@
         <v>525</v>
       </c>
       <c r="AA2" s="25" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="AB2" s="25" t="s">
         <v>526</v>
@@ -24488,7 +24488,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="122.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -24529,7 +24529,7 @@
         <v>386</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H2" s="15" t="s">
         <v>88</v>
@@ -24608,7 +24608,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="121" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="103" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B1" s="104"/>
       <c r="C1" s="104"/>
@@ -24652,7 +24652,7 @@
         <v>97</v>
       </c>
       <c r="G2" s="25" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="H2" s="25" t="s">
         <v>98</v>
@@ -24737,7 +24737,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="126" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -24967,7 +24967,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="30" customFormat="1" ht="173" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="100" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B1" s="101"/>
       <c r="C1" s="101"/>
@@ -24987,13 +24987,13 @@
         <v>2</v>
       </c>
       <c r="D2" s="74" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="E2" s="91" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="F2" s="72" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="G2" s="72" t="s">
         <v>255</v>
@@ -25784,7 +25784,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="110" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="B1" s="101"/>
       <c r="C1" s="101"/>
@@ -25798,7 +25798,7 @@
         <v>87</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>634</v>
@@ -25872,7 +25872,7 @@
         <v>500</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E2" s="25" t="s">
         <v>501</v>
@@ -26259,10 +26259,10 @@
         <v>505</v>
       </c>
       <c r="G2" s="25" t="s">
+        <v>697</v>
+      </c>
+      <c r="H2" s="25" t="s">
         <v>698</v>
-      </c>
-      <c r="H2" s="25" t="s">
-        <v>699</v>
       </c>
       <c r="I2" s="25" t="s">
         <v>100</v>
@@ -26274,7 +26274,7 @@
         <v>266</v>
       </c>
       <c r="L2" s="25" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
   </sheetData>
@@ -26314,7 +26314,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="216" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -26347,10 +26347,10 @@
         <v>507</v>
       </c>
       <c r="D2" s="39" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="F2" s="15" t="s">
         <v>508</v>
@@ -26365,16 +26365,16 @@
         <v>205</v>
       </c>
       <c r="J2" s="15" t="s">
+        <v>801</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>802</v>
+      </c>
+      <c r="L2" s="15" t="s">
         <v>803</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="M2" s="15" t="s">
         <v>804</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>805</v>
-      </c>
-      <c r="M2" s="15" t="s">
-        <v>806</v>
       </c>
       <c r="N2" s="15" t="s">
         <v>509</v>
@@ -26463,7 +26463,7 @@
   <sheetData>
     <row r="1" spans="1:27" s="1" customFormat="1" ht="156" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="103" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B1" s="104"/>
       <c r="C1" s="104"/>
@@ -26503,7 +26503,7 @@
         <v>65</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E2" s="89" t="s">
         <v>448</v>
@@ -32427,7 +32427,7 @@
   <sheetData>
     <row r="1" spans="1:28" s="1" customFormat="1" ht="200.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="114" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B1" s="115"/>
       <c r="C1" s="115"/>
@@ -32467,10 +32467,10 @@
         <v>471</v>
       </c>
       <c r="E2" s="38" t="s">
+        <v>751</v>
+      </c>
+      <c r="F2" s="38" t="s">
         <v>752</v>
-      </c>
-      <c r="F2" s="38" t="s">
-        <v>753</v>
       </c>
       <c r="G2" s="38" t="s">
         <v>450</v>
@@ -36761,7 +36761,7 @@
   <sheetData>
     <row r="1" spans="1:18" ht="138" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="122" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="B1" s="123"/>
       <c r="C1" s="123"/>
@@ -36891,7 +36891,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="52" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="114" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B1" s="123"/>
       <c r="C1" s="123"/>
@@ -36915,7 +36915,7 @@
         <v>641</v>
       </c>
       <c r="C2" s="56" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>652</v>
@@ -36995,7 +36995,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="30" customFormat="1" ht="156.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B1" s="101"/>
       <c r="C1" s="101"/>
@@ -37013,19 +37013,19 @@
         <v>594</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="D2" s="24" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>758</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>759</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>760</v>
-      </c>
       <c r="G2" s="93" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H2" s="24" t="s">
         <v>255</v>
@@ -38121,7 +38121,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="234" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -38130,7 +38130,7 @@
       <c r="F1" s="99"/>
       <c r="G1" s="99"/>
       <c r="H1" s="106" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="I1" s="120"/>
       <c r="J1" s="120"/>
@@ -38145,46 +38145,46 @@
         <v>0</v>
       </c>
       <c r="B2" s="15" t="s">
+        <v>699</v>
+      </c>
+      <c r="C2" s="85" t="s">
         <v>700</v>
       </c>
-      <c r="C2" s="85" t="s">
+      <c r="D2" s="15" t="s">
         <v>701</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="E2" s="15" t="s">
         <v>702</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="F2" s="15" t="s">
+        <v>704</v>
+      </c>
+      <c r="G2" s="38" t="s">
+        <v>705</v>
+      </c>
+      <c r="H2" s="60" t="s">
+        <v>706</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>707</v>
+      </c>
+      <c r="J2" s="86" t="s">
+        <v>708</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>709</v>
+      </c>
+      <c r="L2" s="15" t="s">
+        <v>710</v>
+      </c>
+      <c r="M2" s="87" t="s">
+        <v>711</v>
+      </c>
+      <c r="N2" s="15" t="s">
         <v>703</v>
       </c>
-      <c r="F2" s="15" t="s">
-        <v>705</v>
-      </c>
-      <c r="G2" s="38" t="s">
-        <v>706</v>
-      </c>
-      <c r="H2" s="60" t="s">
-        <v>707</v>
-      </c>
-      <c r="I2" s="15" t="s">
-        <v>708</v>
-      </c>
-      <c r="J2" s="86" t="s">
-        <v>709</v>
-      </c>
-      <c r="K2" s="15" t="s">
-        <v>710</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>711</v>
-      </c>
-      <c r="M2" s="87" t="s">
+      <c r="O2" s="15" t="s">
         <v>712</v>
-      </c>
-      <c r="N2" s="15" t="s">
-        <v>704</v>
-      </c>
-      <c r="O2" s="15" t="s">
-        <v>713</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -39325,7 +39325,7 @@
   <sheetData>
     <row r="1" spans="1:29" ht="212" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="128" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="B1" s="123"/>
       <c r="C1" s="123"/>
@@ -39335,7 +39335,7 @@
       <c r="G1" s="123"/>
       <c r="H1" s="124"/>
       <c r="I1" s="114" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="J1" s="115"/>
       <c r="K1" s="115"/>
@@ -39372,10 +39372,10 @@
         <v>2</v>
       </c>
       <c r="E2" s="96" t="s">
+        <v>771</v>
+      </c>
+      <c r="F2" s="95" t="s">
         <v>772</v>
-      </c>
-      <c r="F2" s="95" t="s">
-        <v>773</v>
       </c>
       <c r="G2" s="96" t="s">
         <v>65</v>
@@ -39384,64 +39384,64 @@
         <v>67</v>
       </c>
       <c r="I2" s="96" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="J2" s="95" t="s">
         <v>66</v>
       </c>
       <c r="K2" s="95" t="s">
+        <v>773</v>
+      </c>
+      <c r="L2" s="95" t="s">
         <v>774</v>
-      </c>
-      <c r="L2" s="95" t="s">
-        <v>775</v>
       </c>
       <c r="M2" s="96" t="s">
         <v>70</v>
       </c>
       <c r="N2" s="96" t="s">
+        <v>775</v>
+      </c>
+      <c r="O2" s="96" t="s">
         <v>776</v>
       </c>
-      <c r="O2" s="96" t="s">
+      <c r="P2" s="96" t="s">
         <v>777</v>
       </c>
-      <c r="P2" s="96" t="s">
+      <c r="Q2" s="96" t="s">
         <v>778</v>
       </c>
-      <c r="Q2" s="96" t="s">
+      <c r="R2" s="96" t="s">
         <v>779</v>
       </c>
-      <c r="R2" s="96" t="s">
+      <c r="S2" s="96" t="s">
         <v>780</v>
       </c>
-      <c r="S2" s="96" t="s">
+      <c r="T2" s="96" t="s">
         <v>781</v>
       </c>
-      <c r="T2" s="96" t="s">
+      <c r="U2" s="96" t="s">
         <v>782</v>
       </c>
-      <c r="U2" s="96" t="s">
+      <c r="V2" s="96" t="s">
         <v>783</v>
       </c>
-      <c r="V2" s="96" t="s">
+      <c r="W2" s="96" t="s">
         <v>784</v>
       </c>
-      <c r="W2" s="96" t="s">
+      <c r="X2" s="96" t="s">
         <v>785</v>
       </c>
-      <c r="X2" s="96" t="s">
+      <c r="Y2" s="96" t="s">
         <v>786</v>
       </c>
-      <c r="Y2" s="96" t="s">
+      <c r="Z2" s="96" t="s">
         <v>787</v>
-      </c>
-      <c r="Z2" s="96" t="s">
-        <v>788</v>
       </c>
       <c r="AA2" s="96" t="s">
         <v>61</v>
       </c>
       <c r="AB2" s="96" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="AC2" s="95" t="s">
         <v>255</v>
@@ -45475,7 +45475,7 @@
   <sheetData>
     <row r="1" spans="1:81" ht="185" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -45501,13 +45501,13 @@
         <v>2</v>
       </c>
       <c r="E2" s="24" t="s">
+        <v>790</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>791</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="G2" s="24" t="s">
         <v>792</v>
-      </c>
-      <c r="G2" s="24" t="s">
-        <v>793</v>
       </c>
       <c r="H2" s="24" t="s">
         <v>255</v>
@@ -48607,7 +48607,7 @@
       </c>
       <c r="F38" s="44"/>
       <c r="G38" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="H38" s="44"/>
       <c r="I38" s="44"/>
@@ -48643,7 +48643,7 @@
     <row r="39" spans="1:35" s="43" customFormat="1" x14ac:dyDescent="0.2">
       <c r="F39" s="44"/>
       <c r="G39" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H39" s="44"/>
       <c r="I39" s="44"/>
@@ -50339,7 +50339,7 @@
   <sheetData>
     <row r="1" spans="1:6" s="30" customFormat="1" ht="131.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B1" s="101"/>
       <c r="C1" s="101"/>
@@ -51939,7 +51939,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="30" customFormat="1" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B1" s="99"/>
       <c r="C1" s="99"/>
@@ -54431,7 +54431,7 @@
   <sheetData>
     <row r="1" spans="1:14" s="30" customFormat="1" ht="207" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B1" s="101"/>
       <c r="C1" s="101"/>

</xml_diff>

<commit_message>
Automation Toolkit Release v2025.2.1
</commit_message>
<xml_diff>
--- a/cd3_automation_toolkit/example/CD3-Blank-template.xlsx
+++ b/cd3_automation_toolkit/example/CD3-Blank-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/susingla/PycharmProjects/orahub-develop/cd3_automation_toolkit/example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B0B012-7156-6549-9B5A-42C408225E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA357495-56B2-2F44-9949-7C24D9C27283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="28800" windowHeight="17400" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -835,7 +835,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="821">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="822">
   <si>
     <t>Region</t>
   </si>
@@ -11343,6 +11343,9 @@
       <t xml:space="preserve">
 Updated Instances sheet, Exa-Infra sheet</t>
     </r>
+  </si>
+  <si>
+    <t>Plugin OS Management Service Agent</t>
   </si>
 </sst>
 </file>
@@ -23760,7 +23763,7 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:AJ2"/>
+  <dimension ref="A1:AK2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
@@ -23786,11 +23789,12 @@
     <col min="21" max="21" width="13.1640625" hidden="1" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" hidden="1" customWidth="1"/>
     <col min="23" max="29" width="0" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="15" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="15" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="311" customHeight="1">
+    <row r="1" spans="1:37" ht="311" customHeight="1">
       <c r="A1" s="114" t="s">
         <v>767</v>
       </c>
@@ -23830,9 +23834,10 @@
       <c r="AG1" s="101"/>
       <c r="AH1" s="101"/>
       <c r="AI1" s="101"/>
-      <c r="AJ1" s="102"/>
-    </row>
-    <row r="2" spans="1:36" s="30" customFormat="1" ht="83.25" customHeight="1">
+      <c r="AJ1" s="101"/>
+      <c r="AK1" s="102"/>
+    </row>
+    <row r="2" spans="1:37" s="30" customFormat="1" ht="83.25" customHeight="1">
       <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
@@ -23918,34 +23923,37 @@
         <v>818</v>
       </c>
       <c r="AC2" s="25" t="s">
+        <v>821</v>
+      </c>
+      <c r="AD2" s="25" t="s">
         <v>819</v>
       </c>
-      <c r="AD2" s="24" t="s">
+      <c r="AE2" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="AE2" s="24" t="s">
+      <c r="AF2" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="AF2" s="25" t="s">
+      <c r="AG2" s="25" t="s">
         <v>373</v>
       </c>
-      <c r="AG2" s="24" t="s">
+      <c r="AH2" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="AH2" s="25" t="s">
+      <c r="AI2" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="AI2" s="25" t="s">
+      <c r="AJ2" s="25" t="s">
         <v>636</v>
       </c>
-      <c r="AJ2" s="24" t="s">
+      <c r="AK2" s="24" t="s">
         <v>255</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:AJ1"/>
+    <mergeCell ref="I1:AK1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="1" sqref="D1:D1048576 H3:P1048576 S3:XFD1048576 E1:XFD2 A1:C2" xr:uid="{70506928-0DD3-F44D-BCEE-021DFE2CA7EA}"/>

</xml_diff>